<commit_message>
more stuff and things
</commit_message>
<xml_diff>
--- a/results/classifications.xlsx
+++ b/results/classifications.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -558,6 +558,33 @@
       </c>
       <c r="I2" t="n">
         <v>39.53126083291136</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>meta-llama/Llama-3.2-1B-Instruct</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="n">
+        <v>167.5189627920045</v>
       </c>
     </row>
   </sheetData>

</xml_diff>